<commit_message>
Fix tecnologies errors and coordinates errors
</commit_message>
<xml_diff>
--- a/arquivos/id_tecnologia_facilidades.xlsx
+++ b/arquivos/id_tecnologia_facilidades.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\F257064\Documents\Codes\atualizacao automacao lote\AUTMACAO_LOTE\arquivos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D1F90B8-9988-4E2E-A2AB-E2CE97098F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D3B701-1004-4501-ABDB-9D00383EDAC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="62">
   <si>
     <t>FACILIDADE</t>
   </si>
@@ -203,9 +203,6 @@
     <t>RADIO IP</t>
   </si>
   <si>
-    <t>FO GPON_RESID ETH PV</t>
-  </si>
-  <si>
     <t>BANDA KA</t>
   </si>
   <si>
@@ -222,6 +219,9 @@
   </si>
   <si>
     <t>LTE(4G)</t>
+  </si>
+  <si>
+    <t>TERCEIRO SIMÉTRICO</t>
   </si>
 </sst>
 </file>
@@ -539,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="30.5546875" bestFit="1" customWidth="1"/>
@@ -584,10 +584,10 @@
         <v>3</v>
       </c>
       <c r="E2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G2">
         <v>8</v>
@@ -610,7 +610,7 @@
         <v>33</v>
       </c>
       <c r="F3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G3">
         <v>8</v>
@@ -633,7 +633,7 @@
         <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G4">
         <v>8</v>
@@ -656,7 +656,7 @@
         <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G5">
         <v>8</v>
@@ -679,7 +679,7 @@
         <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G6">
         <v>8</v>
@@ -702,7 +702,7 @@
         <v>35</v>
       </c>
       <c r="F7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G7">
         <v>8</v>
@@ -722,10 +722,10 @@
         <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="F8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G8">
         <v>8</v>
@@ -745,7 +745,7 @@
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G9">
         <v>8</v>
@@ -768,7 +768,7 @@
         <v>7</v>
       </c>
       <c r="F10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G10">
         <v>8</v>
@@ -791,7 +791,7 @@
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G11">
         <v>8</v>
@@ -814,7 +814,7 @@
         <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G12">
         <v>8</v>
@@ -837,7 +837,7 @@
         <v>11</v>
       </c>
       <c r="F13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G13">
         <v>8</v>
@@ -860,7 +860,7 @@
         <v>13</v>
       </c>
       <c r="F14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G14">
         <v>8</v>
@@ -883,7 +883,7 @@
         <v>15</v>
       </c>
       <c r="F15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G15">
         <v>8</v>
@@ -906,7 +906,7 @@
         <v>40</v>
       </c>
       <c r="F16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G16">
         <v>8</v>
@@ -929,7 +929,7 @@
         <v>53</v>
       </c>
       <c r="F17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G17">
         <v>8</v>
@@ -952,7 +952,7 @@
         <v>41</v>
       </c>
       <c r="F18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G18">
         <v>8</v>
@@ -975,7 +975,7 @@
         <v>42</v>
       </c>
       <c r="F19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G19">
         <v>8</v>
@@ -992,10 +992,10 @@
         <v>39</v>
       </c>
       <c r="E20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G20">
         <v>8</v>
@@ -1012,10 +1012,10 @@
         <v>39</v>
       </c>
       <c r="E21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G21">
         <v>8</v>
@@ -1038,7 +1038,7 @@
         <v>52</v>
       </c>
       <c r="F22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G22">
         <v>8</v>
@@ -1061,7 +1061,7 @@
         <v>45</v>
       </c>
       <c r="F23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G23">
         <v>8</v>
@@ -1078,7 +1078,7 @@
         <v>46</v>
       </c>
       <c r="E24" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -1092,26 +1092,40 @@
         <v>46</v>
       </c>
       <c r="E25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
+        <v>26</v>
+      </c>
+      <c r="B26" t="s">
+        <v>29</v>
+      </c>
+      <c r="D26" t="s">
+        <v>46</v>
+      </c>
+      <c r="E26" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27">
         <v>21</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>31</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D27" t="s">
         <v>49</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E27" t="s">
         <v>54</v>
       </c>
-      <c r="F26" t="s">
-        <v>58</v>
-      </c>
-      <c r="G26">
+      <c r="F27" t="s">
+        <v>57</v>
+      </c>
+      <c r="G27">
         <v>8</v>
       </c>
     </row>

</xml_diff>